<commit_message>
Update rugby league data
</commit_message>
<xml_diff>
--- a/src/data/superLeagueMatches.xlsx
+++ b/src/data/superLeagueMatches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\acann\rugby-league-supporter-web\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B301E35-3324-42DA-B5B7-1D891021C7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F70CAB9-0484-4634-8C10-8A7E64F67B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13215" yWindow="-16395" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="979" uniqueCount="52">
   <si>
     <t>Date</t>
   </si>
@@ -176,9 +176,6 @@
   </si>
   <si>
     <t>To be confirmed</t>
-  </si>
-  <si>
-    <t>LIVE</t>
   </si>
 </sst>
 </file>
@@ -3722,17 +3719,11 @@
       <c r="C127" t="s">
         <v>26</v>
       </c>
-      <c r="D127">
-        <v>2</v>
-      </c>
-      <c r="E127">
-        <v>0</v>
-      </c>
       <c r="F127" t="s">
         <v>28</v>
       </c>
       <c r="G127" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
       <c r="H127" t="s">
         <v>35</v>

</xml_diff>